<commit_message>
Add support for histogram
</commit_message>
<xml_diff>
--- a/20240229_oliynyk_test_atom_mixing_formatted/output/20240229_oliynyk_test_atom_mixing_formatted_pairs.xlsx
+++ b/20240229_oliynyk_test_atom_mixing_formatted/output/20240229_oliynyk_test_atom_mixing_formatted_pairs.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-Ga (1)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ga-Ga (1)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ga-La (1)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-Ga" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ga-Ga" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ga-La" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,6 +438,11 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Atomic Site</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Distance</t>
         </is>
       </c>
@@ -448,7 +453,8 @@
           <t>539016.cif</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="n">
         <v>2.601</v>
       </c>
     </row>
@@ -463,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +480,11 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Atomic Site</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Distance</t>
         </is>
       </c>
@@ -484,7 +495,8 @@
           <t>539016.cif</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="n">
         <v>2.601</v>
       </c>
     </row>
@@ -499,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +522,11 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Atomic Site</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Distance</t>
         </is>
       </c>
@@ -520,7 +537,8 @@
           <t>539016.cif</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="n">
         <v>3.291</v>
       </c>
     </row>

</xml_diff>